<commit_message>
feat: seletor híbrido com diagnóstico de recall de limitações; regra de confiança v2 (categórica); notebook reutiliza execuções gravadas
- select: HybridSelector (semântica + seções finais + janelas de pista), recall_table, keyword com cabeçalhos de fechamento
- audit: ConfidenceRule(input_effect_mode) com RULE_V1/RULE_V2, confidence_by_rule; ADR 0005 com a calibração medida
- notebook: FICHA_REUSAR/FICHA_ESTRATEGIA, v1 × v2 lado a lado, achados reais (vazamento do few-shot, páginas erradas)
- 374 testes passando

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/outputs/AtividadeI_Mascena_Lira_Murakami_Garbin.xlsx
+++ b/data/outputs/AtividadeI_Mascena_Lira_Murakami_Garbin.xlsx
@@ -533,12 +533,12 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>baixa</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>6 campos mudaram entre estratégias de entrada (instável)</t>
+          <t>trecho encontrado (exact, score 1.00) na página declarada p. 10; estável entre repetições e estratégias</t>
         </is>
       </c>
     </row>
@@ -579,12 +579,12 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2 campo(s) mudou(aram) entre estratégias de entrada</t>
+          <t>trecho encontrado (exact, score 1.00) na página declarada p. 2; estável entre repetições e estratégias</t>
         </is>
       </c>
     </row>
@@ -625,12 +625,12 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2 campo(s) mudou(aram) entre estratégias de entrada</t>
+          <t>trecho encontrado (exact, score 1.00) na página declarada p. 2; estável entre repetições e estratégias</t>
         </is>
       </c>
     </row>
@@ -671,12 +671,12 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>baixa</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>4 campos mudaram entre estratégias de entrada (instável)</t>
+          <t>trecho encontrado (exact, score 1.00) na página declarada p. 3; estável entre repetições e estratégias</t>
         </is>
       </c>
     </row>
@@ -717,12 +717,12 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>baixa</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>6 campos mudaram entre estratégias de entrada (instável)</t>
+          <t>trecho encontrado (exact, score 1.00) na página declarada p. 15; estável entre repetições e estratégias</t>
         </is>
       </c>
     </row>
@@ -768,7 +768,7 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>trecho não encontrado no texto enviado (score 0.47 &lt; 0.90): possível trecho inventado; 6 campos mudaram entre estratégias de entrada (instável)</t>
+          <t>trecho não encontrado no texto enviado (score 0.47 &lt; 0.90): possível trecho inventado</t>
         </is>
       </c>
     </row>
@@ -809,12 +809,12 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>baixa</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>6 campos mudaram entre estratégias de entrada (instável)</t>
+          <t>trecho encontrado (exact, score 1.00) na página declarada p. 55; estável entre repetições e estratégias</t>
         </is>
       </c>
     </row>
@@ -860,7 +860,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>página errada: declarada p. 15, trecho localizado em p. 16; 6 campos mudaram entre estratégias de entrada (instável)</t>
+          <t>página errada: declarada p. 15, trecho localizado em p. 16</t>
         </is>
       </c>
     </row>
@@ -901,12 +901,12 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>baixa</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>6 campos mudaram entre estratégias de entrada (instável)</t>
+          <t>trecho encontrado (exact, score 1.00) na página declarada p. 5; estável entre repetições e estratégias</t>
         </is>
       </c>
     </row>
@@ -947,12 +947,12 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>baixa</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>6 campos mudaram entre estratégias de entrada (instável)</t>
+          <t>trecho encontrado (exact, score 1.00) na página declarada p. 4; estável entre repetições e estratégias</t>
         </is>
       </c>
     </row>
@@ -993,12 +993,12 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>baixa</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>6 campos mudaram entre estratégias de entrada (instável)</t>
+          <t>trecho encontrado (exact, score 1.00) na página declarada p. 9; estável entre repetições e estratégias</t>
         </is>
       </c>
     </row>
@@ -1039,12 +1039,12 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>baixa</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>6 campos mudaram entre estratégias de entrada (instável)</t>
+          <t>trecho encontrado (exact, score 1.00) na página declarada p. 1; estável entre repetições e estratégias</t>
         </is>
       </c>
     </row>
@@ -1085,12 +1085,12 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>baixa</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>6 campos mudaram entre estratégias de entrada (instável)</t>
+          <t>trecho encontrado (exact, score 1.00) na página declarada p. 13; estável entre repetições e estratégias</t>
         </is>
       </c>
     </row>
@@ -1131,12 +1131,12 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>baixa</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>6 campos mudaram entre estratégias de entrada (instável)</t>
+          <t>trecho encontrado (exact, score 1.00) na página declarada p. 18; estável entre repetições e estratégias</t>
         </is>
       </c>
     </row>
@@ -1181,12 +1181,12 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>baixa</t>
+          <t>media</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>7 campos mudaram entre estratégias de entrada (instável)</t>
+          <t>discordância categórica entre estratégias de entrada: limitacao é null numa e preenchida na outra</t>
         </is>
       </c>
     </row>
@@ -1227,12 +1227,12 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>baixa</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>6 campos mudaram entre estratégias de entrada (instável)</t>
+          <t>trecho encontrado (exact, score 1.00) na página declarada p. 8; estável entre repetições e estratégias</t>
         </is>
       </c>
     </row>
@@ -1273,12 +1273,12 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>baixa</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>5 campos mudaram entre estratégias de entrada (instável)</t>
+          <t>trecho encontrado (exact, score 1.00) na página declarada p. 1; estável entre repetições e estratégias</t>
         </is>
       </c>
     </row>
@@ -1319,12 +1319,12 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>baixa</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>6 campos mudaram entre estratégias de entrada (instável)</t>
+          <t>trecho encontrado (fuzzy, score 0.98) na página declarada p. 12; estável entre repetições e estratégias</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>página errada: declarada p. 18, trecho localizado em p. 15; 6 campos mudaram entre estratégias de entrada (instável)</t>
+          <t>página errada: declarada p. 18, trecho localizado em p. 15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: entregáveis finais — notebook real (semantic), tabela, relatório de 3 páginas; experimento híbrido documentado
- estratégia final semantic pelo critério declarado (página correta 16/19); hybrid medido e descartado
- verificação e) vazamento de exemplos no notebook e no PDF; regra v2: alta 14 / média 1 / baixa 4
- custo real US$ 1,88 (117 chamadas) vs US$ 8,28 ingênuo (4,4×)
- run hybrid rep2 interrompido em 16/19 e marcado no manifesto; títulos do PDF com keepWithNext
- 394 testes passando

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/outputs/AtividadeI_Mascena_Lira_Murakami_Garbin.xlsx
+++ b/data/outputs/AtividadeI_Mascena_Lira_Murakami_Garbin.xlsx
@@ -768,7 +768,7 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>trecho não encontrado no texto enviado (score 0.47 &lt; 0.90): possível trecho inventado</t>
+          <t>campo dados copiado do exemplo few-shot (similaridade 0.97); campo metodo copiado do exemplo few-shot (similaridade 1.00); campo metrica copiado do exemplo few-shot (similaridade 1.00); campo evidencia.trecho copiado do exemplo few-shot (similaridade 1.00); campo dados contém 'supermercados', 'vendas', termos do exemplo few-shot ausentes do texto enviado; campo metodo contém 'promoções', 'feriados', termos do exemplo few-shot ausentes do texto enviado; campo metrica contém 'WMAPE', 'suavização exponencial', termos do exemplo few-shot ausentes do texto enviado; campo evidencia.trecho contém 'WMAPE', termo do exemplo few-shot ausente do texto enviado; trecho não encontrado no texto enviado (score 0.47 &lt; 0.90): possível trecho inventado</t>
         </is>
       </c>
     </row>
@@ -809,12 +809,12 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>alta</t>
+          <t>baixa</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>trecho encontrado (exact, score 1.00) na página declarada p. 55; estável entre repetições e estratégias</t>
+          <t>campo dados contém 'supermercados', termo do exemplo few-shot ausente do texto enviado</t>
         </is>
       </c>
     </row>

</xml_diff>